<commit_message>
Updated the InventoryFormClass, Added the test for it
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/TestData.xlsx
+++ b/src/test/java/TestData/TestData.xlsx
@@ -1,108 +1,50 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Ndosi Test\AdvacedFormAutomaton\src\test\java\TestData\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{022AAC39-6F04-4714-85BF-CCF86A00C5C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-16320" yWindow="-120" windowWidth="16440" windowHeight="28320" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-16320" yWindow="-120" windowWidth="16440" windowHeight="28320" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Information Tab" sheetId="2" r:id="rId1"/>
-    <sheet name="Login Details" sheetId="1" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Information Tab" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login Details" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory Details" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
-  <si>
-    <t>Username</t>
-  </si>
-  <si>
-    <t>Password</t>
-  </si>
-  <si>
-    <t>secret_sauce</t>
-  </si>
-  <si>
-    <t>locked_out_user</t>
-  </si>
-  <si>
-    <t>problem_user</t>
-  </si>
-  <si>
-    <t>Cele</t>
-  </si>
-  <si>
-    <t>Nkosi</t>
-  </si>
-  <si>
-    <t>@12345678</t>
-  </si>
-  <si>
-    <t>wrongPassword</t>
-  </si>
-  <si>
-    <t>test@gmail.com</t>
-  </si>
-  <si>
-    <t>nolo@test.com</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="10"/>
+      <sz val="11"/>
+      <u val="single"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.59999389629810485"/>
+        <fgColor theme="4" tint="0.5999938962981048"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -139,29 +81,88 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="5">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="1" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -427,81 +428,189 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21EDF707-6210-4854-82A6-DC939659F70F}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="17" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.140625" bestFit="1" customWidth="1"/>
+    <col width="17" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="14.140625" bestFit="1" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1" t="s">
-        <v>6</v>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Username</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Password</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>nolo@test.com</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>@12345678</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>locked_out_user</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>secret_sauce</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>problem_user</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>wrongPassword</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="n"/>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>Cele</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>test@gmail.com</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>secret_sauce</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n"/>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>Nkosi</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" display="password@1" xr:uid="{DB7CB863-1276-44F8-BEBF-77A1C5D85F49}"/>
-    <hyperlink ref="A6" r:id="rId2" xr:uid="{D7A13239-1DDF-4FE9-8D01-E2B21D846603}"/>
-    <hyperlink ref="A2" r:id="rId3" xr:uid="{AE642B6E-A097-4D4C-AE94-9C75591F73B4}"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" display="password@1" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>DeviceType</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Storage</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Colour</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>128GB</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>123 Test Street</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
updated the extras page to include the click purchase button
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/TestData.xlsx
+++ b/src/test/java/TestData/TestData.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Ndosi Test\AdvacedFormAutomaton\src\test\java\TestData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Twins\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_2924184101AEFC028C932E4858E71FC1C998FEEE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19B5A7EC-D9C8-4659-847C-1FFAD94674CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-16320" yWindow="-120" windowWidth="16440" windowHeight="28320" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Information Tab" sheetId="1" r:id="rId1"/>
@@ -73,9 +73,6 @@
     <t>express</t>
   </si>
   <si>
-    <t>2yr</t>
-  </si>
-  <si>
     <t>SAVE10</t>
   </si>
   <si>
@@ -113,6 +110,9 @@
   </si>
   <si>
     <t>123 Test Street</t>
+  </si>
+  <si>
+    <t>1yr</t>
   </si>
 </sst>
 </file>
@@ -573,13 +573,13 @@
         <v>15</v>
       </c>
       <c r="B2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" t="s">
         <v>16</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>17</v>
-      </c>
-      <c r="D2" t="s">
-        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -594,42 +594,42 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" t="s">
         <v>19</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>20</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>21</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>22</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>23</v>
-      </c>
-      <c r="F1" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
         <v>25</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>26</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>27</v>
-      </c>
-      <c r="D2" t="s">
-        <v>28</v>
       </c>
       <c r="E2">
         <v>2</v>
       </c>
       <c r="F2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>